<commit_message>
chore: update remaining print pack templates
</commit_message>
<xml_diff>
--- a/data/print_templates/B__packing_list_carton__per_carton_single.xlsx
+++ b/data/print_templates/B__packing_list_carton__per_carton_single.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/EdouardGonnu/asf-wms/data/print_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7659606F-A33D-1842-BA15-66F3C06CAC45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355159CE-9307-BF49-B04A-ED59E4CC4AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{D41FDF60-E254-7C4C-BFC3-DDF9FE3B5742}"/>
+    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16940" xr2:uid="{D41FDF60-E254-7C4C-BFC3-DDF9FE3B5742}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$D$18</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -44,12 +44,6 @@
     <t>QUANTITE</t>
   </si>
   <si>
-    <t>Dons humanitaires non destinés à être revendus - Produits non dangereux</t>
-  </si>
-  <si>
-    <t>FORME</t>
-  </si>
-  <si>
     <t>PRODUIT</t>
   </si>
   <si>
@@ -58,12 +52,19 @@
   <si>
     <t>Référence du colis :</t>
   </si>
+  <si>
+    <t>Dons humanitaires non destinés à être revendus
+Produits non dangereux</t>
+  </si>
+  <si>
+    <t>LISTE DE COLISAGE</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -84,6 +85,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -99,7 +107,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -123,7 +131,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -137,9 +147,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -151,47 +159,12 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -222,7 +195,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -233,44 +206,37 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="7">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
@@ -309,21 +275,6 @@
         <left style="thin">
           <color indexed="64"/>
         </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
         <right style="thin">
           <color indexed="64"/>
         </right>
@@ -415,25 +366,20 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1689100</xdr:colOff>
+      <xdr:colOff>381000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>419100</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>83139</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="968000" cy="589817"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 2">
+        <xdr:cNvPr id="2" name="Image 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C9C4F77-CF54-4ACB-1345-D62F0FF6B5F5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{383A08E9-672A-C440-8FC4-2648DB93F9E7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -441,22 +387,15 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect t="18570" b="15109"/>
+        <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1689100" y="63500"/>
-          <a:ext cx="4025900" cy="1238839"/>
+          <a:off x="381000" y="127000"/>
+          <a:ext cx="968000" cy="589817"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -464,15 +403,14 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{86EF37FB-E506-1E4C-98B6-94A9E27D3858}" name="Tableau2" displayName="Tableau2" ref="A10:D20" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
-  <autoFilter ref="A10:D20" xr:uid="{86EF37FB-E506-1E4C-98B6-94A9E27D3858}"/>
-  <tableColumns count="4">
-    <tableColumn id="2" xr3:uid="{BBFB573B-AD59-804B-B19E-5E817460BD0B}" name="FORME" dataDxfId="3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{86EF37FB-E506-1E4C-98B6-94A9E27D3858}" name="Tableau2" displayName="Tableau2" ref="A7:C17" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
+  <autoFilter ref="A7:C17" xr:uid="{86EF37FB-E506-1E4C-98B6-94A9E27D3858}"/>
+  <tableColumns count="3">
     <tableColumn id="3" xr3:uid="{FBFF4320-0029-1F4A-80B8-9873748E956F}" name="PRODUIT" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{6694315A-10C9-2A4F-9F6E-2A7012ED73F4}" name="QUANTITE" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{3957F165-746F-D343-A9EF-25CE93FC4BC3}" name="DATE LIMITE" dataDxfId="0"/>
@@ -801,134 +739,102 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:D20"/>
+  <dimension ref="A2:C17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="23.1640625" customWidth="1"/>
-    <col min="5" max="5" width="2.83203125" customWidth="1"/>
+    <col min="1" max="3" width="23.1640625" customWidth="1"/>
+    <col min="4" max="4" width="2.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="14"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="14"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="14"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-    </row>
-    <row r="8" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="13" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="11"/>
+      <c r="B2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="13"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="5" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>5</v>
+      <c r="B7" s="2" t="s">
+        <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="9"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="11"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="9"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="11"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="9"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="11"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="11"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="11"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="9"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="11"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="9"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="11"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="9"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="11"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="10"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="12"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="6"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="8"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="6"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="8"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="6"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="8"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="6"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="8"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="6"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="8"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="6"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="8"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="6"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="8"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="6"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="8"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="6"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="8"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="7"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A2:D6"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="B2:C3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="11" scale="86" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>